<commit_message>
passage au thème et au makefile
</commit_message>
<xml_diff>
--- a/template/horaire-rencontre.xlsx
+++ b/template/horaire-rencontre.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/techno/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E575B3-56AC-0943-9075-F482EABB1DD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D4E8E9-B5C9-524C-A126-BF42CFF90117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{B002BC29-BF88-984D-8C72-1939D715F278}"/>
   </bookViews>
   <sheets>
-    <sheet name="grille" sheetId="1" r:id="rId1"/>
+    <sheet name="horaire" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ListeEtudiants_cours4205A3VI_gr00001" localSheetId="0">grille!$A$2:$C$26</definedName>
+    <definedName name="ListeEtudiants_cours4205A3VI_gr00001" localSheetId="0">horaire!$A$2:$C$26</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -559,7 +559,7 @@
         <v>15</v>
       </c>
       <c r="C3" s="1">
-        <f>C2+C$27</f>
+        <f t="shared" ref="C3:C15" si="0">C2+C$27</f>
         <v>45994.602083333331</v>
       </c>
     </row>
@@ -571,7 +571,7 @@
         <v>24</v>
       </c>
       <c r="C4" s="1">
-        <f>C3+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.610416666663</v>
       </c>
     </row>
@@ -583,7 +583,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="1">
-        <f>C4+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.618749999994</v>
       </c>
     </row>
@@ -595,7 +595,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1">
-        <f>C5+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.627083333326</v>
       </c>
     </row>
@@ -607,7 +607,7 @@
         <v>23</v>
       </c>
       <c r="C7" s="1">
-        <f>C6+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.635416666657</v>
       </c>
     </row>
@@ -619,7 +619,7 @@
         <v>13</v>
       </c>
       <c r="C8" s="1">
-        <f>C7+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.643749999988</v>
       </c>
     </row>
@@ -631,7 +631,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="1">
-        <f>C8+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.65208333332</v>
       </c>
     </row>
@@ -643,7 +643,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="1">
-        <f>C9+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.660416666651</v>
       </c>
     </row>
@@ -655,7 +655,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="1">
-        <f>C10+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.668749999983</v>
       </c>
     </row>
@@ -667,7 +667,7 @@
         <v>26</v>
       </c>
       <c r="C12" s="1">
-        <f>C11+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.677083333314</v>
       </c>
     </row>
@@ -679,7 +679,7 @@
         <v>4</v>
       </c>
       <c r="C13" s="1">
-        <f>C12+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.685416666645</v>
       </c>
     </row>
@@ -691,7 +691,7 @@
         <v>12</v>
       </c>
       <c r="C14" s="1">
-        <f>C13+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.693749999977</v>
       </c>
     </row>
@@ -703,7 +703,7 @@
         <v>11</v>
       </c>
       <c r="C15" s="1">
-        <f>C14+C$27</f>
+        <f t="shared" si="0"/>
         <v>45994.702083333308</v>
       </c>
     </row>
@@ -726,7 +726,7 @@
         <v>25</v>
       </c>
       <c r="C17" s="1">
-        <f>C16+C$27</f>
+        <f t="shared" ref="C17:C26" si="1">C16+C$27</f>
         <v>46001.602083333331</v>
       </c>
     </row>
@@ -738,7 +738,7 @@
         <v>10</v>
       </c>
       <c r="C18" s="1">
-        <f>C17+C$27</f>
+        <f t="shared" si="1"/>
         <v>46001.610416666663</v>
       </c>
     </row>
@@ -750,7 +750,7 @@
         <v>14</v>
       </c>
       <c r="C19" s="1">
-        <f>C18+C$27</f>
+        <f t="shared" si="1"/>
         <v>46001.618749999994</v>
       </c>
     </row>
@@ -762,7 +762,7 @@
         <v>9</v>
       </c>
       <c r="C20" s="1">
-        <f>C19+C$27</f>
+        <f t="shared" si="1"/>
         <v>46001.627083333326</v>
       </c>
     </row>
@@ -774,7 +774,7 @@
         <v>2</v>
       </c>
       <c r="C21" s="1">
-        <f>C20+C$27</f>
+        <f t="shared" si="1"/>
         <v>46001.635416666657</v>
       </c>
     </row>
@@ -786,7 +786,7 @@
         <v>22</v>
       </c>
       <c r="C22" s="1">
-        <f>C21+C$27</f>
+        <f t="shared" si="1"/>
         <v>46001.643749999988</v>
       </c>
     </row>
@@ -798,7 +798,7 @@
         <v>3</v>
       </c>
       <c r="C23" s="1">
-        <f>C22+C$27</f>
+        <f t="shared" si="1"/>
         <v>46001.65208333332</v>
       </c>
     </row>
@@ -810,7 +810,7 @@
         <v>18</v>
       </c>
       <c r="C24" s="1">
-        <f>C23+C$27</f>
+        <f t="shared" si="1"/>
         <v>46001.660416666651</v>
       </c>
     </row>
@@ -822,7 +822,7 @@
         <v>6</v>
       </c>
       <c r="C25" s="1">
-        <f>C24+C$27</f>
+        <f t="shared" si="1"/>
         <v>46001.668749999983</v>
       </c>
     </row>
@@ -834,7 +834,7 @@
         <v>17</v>
       </c>
       <c r="C26" s="1">
-        <f>C25+C$27</f>
+        <f t="shared" si="1"/>
         <v>46001.677083333314</v>
       </c>
     </row>

</xml_diff>